<commit_message>
Création TU pour le Cas S02
</commit_message>
<xml_diff>
--- a/Manuel Validation/CAS S04/Cas S04.xlsx
+++ b/Manuel Validation/CAS S04/Cas S04.xlsx
@@ -57,6 +57,7 @@
     <definedName name="MEd_U2">'S04'!$J$25</definedName>
     <definedName name="MEdG">'S04'!$J$13</definedName>
     <definedName name="MelRd">'S04'!$Q$27</definedName>
+    <definedName name="MfRd">'S04'!$Q$45</definedName>
     <definedName name="MplRd">'S04'!$Q$43</definedName>
     <definedName name="MRd">'S04'!$E$50</definedName>
     <definedName name="MStatS">'S04'!$E$79</definedName>
@@ -95,7 +96,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="147">
   <si>
     <t xml:space="preserve">PRS </t>
   </si>
@@ -527,6 +528,15 @@
   </si>
   <si>
     <t>Nidi</t>
+  </si>
+  <si>
+    <t>MfRd</t>
+  </si>
+  <si>
+    <t>GMvB</t>
+  </si>
+  <si>
+    <t>Plastique</t>
   </si>
 </sst>
 </file>
@@ -960,9 +970,6 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="1" fontId="0" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1001,6 +1008,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1354,7 +1364,7 @@
         <v>134</v>
       </c>
       <c r="I7" s="6">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="J7" t="s">
         <v>12</v>
@@ -1518,7 +1528,7 @@
       </c>
       <c r="J15" s="9">
         <f>-qQ_1*La^2/2</f>
-        <v>-312.5</v>
+        <v>-375</v>
       </c>
       <c r="K15" s="18" t="s">
         <v>23</v>
@@ -1550,7 +1560,7 @@
       </c>
       <c r="J16" s="8">
         <f>qQ_1*La</f>
-        <v>250</v>
+        <v>300</v>
       </c>
       <c r="K16" s="21" t="s">
         <v>13</v>
@@ -1756,7 +1766,7 @@
       </c>
       <c r="J23" s="8">
         <f>GammaG*MEdG+GammaQ*(MEd_Q1+Psi_0*MEd_Q2)</f>
-        <v>-312.5</v>
+        <v>-375</v>
       </c>
       <c r="K23" s="31" t="s">
         <v>23</v>
@@ -1779,7 +1789,7 @@
       </c>
       <c r="J24" s="8">
         <f>GammaG*VEdG+GammaQ*(VEd_Q1+Psi_0*VEd_Q2)</f>
-        <v>250</v>
+        <v>300</v>
       </c>
       <c r="K24" s="34" t="s">
         <v>13</v>
@@ -1813,7 +1823,7 @@
       </c>
       <c r="J25" s="8">
         <f>GammaG*MEdG+GammaQ*(Psi_0*MEd_Q1+MEd_Q2)</f>
-        <v>-218.75</v>
+        <v>-262.5</v>
       </c>
       <c r="K25" s="37" t="s">
         <v>23</v>
@@ -1821,7 +1831,7 @@
       <c r="M25" s="50" t="s">
         <v>108</v>
       </c>
-      <c r="N25" s="8">
+      <c r="N25" s="55">
         <f>SUM(R21:S21)</f>
         <v>143293261.26126125</v>
       </c>
@@ -1831,7 +1841,7 @@
       <c r="P25" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="Q25" s="70">
+      <c r="Q25" s="69">
         <f>InertieCM4/(ABS(zG))*10</f>
         <v>838.10475287174631</v>
       </c>
@@ -1848,12 +1858,12 @@
       </c>
       <c r="J26" s="8">
         <f>GammaG*VEdG+GammaQ*(Psi_0*VEd_Q1+VEd_Q2)</f>
-        <v>175</v>
+        <v>210</v>
       </c>
       <c r="K26" s="40" t="s">
         <v>13</v>
       </c>
-      <c r="N26" s="8">
+      <c r="N26" s="55">
         <f>N25/10^4</f>
         <v>14329.326126126125</v>
       </c>
@@ -1863,7 +1873,7 @@
       <c r="P26" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="Q26" s="70">
+      <c r="Q26" s="69">
         <f>InertieCM4/(Ht-ABS(zG))*10</f>
         <v>961.52532946439351</v>
       </c>
@@ -1877,7 +1887,7 @@
       <c r="P27" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="Q27" s="64">
+      <c r="Q27" s="63">
         <f>MIN(Q25*FyS,Q26*FyI)/1000/GammaM0</f>
         <v>385.52818632100332</v>
       </c>
@@ -1910,7 +1920,7 @@
       </c>
       <c r="J30" s="5">
         <f>GammaG*qG+GammaQ*qQ_1</f>
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="K30" t="s">
         <v>12</v>
@@ -1941,12 +1951,12 @@
       </c>
     </row>
     <row r="32" spans="3:19" x14ac:dyDescent="0.25">
-      <c r="C32" s="65" t="s">
+      <c r="C32" s="64" t="s">
         <v>64</v>
       </c>
-      <c r="D32" s="65"/>
-      <c r="E32" s="65"/>
-      <c r="F32" s="65"/>
+      <c r="D32" s="64"/>
+      <c r="E32" s="64"/>
+      <c r="F32" s="64"/>
       <c r="M32" s="3" t="s">
         <v>53</v>
       </c>
@@ -1985,9 +1995,9 @@
       <c r="R33" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="S33" s="73">
+      <c r="S33" s="72">
         <f>IF(E60&gt;0.5,(2*E60-1)^2,0)</f>
-        <v>1.4552389804685017E-2</v>
+        <v>0.11885941882460893</v>
       </c>
     </row>
     <row r="34" spans="3:22" x14ac:dyDescent="0.25">
@@ -2014,7 +2024,7 @@
       <c r="R34" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="S34" s="73">
+      <c r="S34" s="72">
         <f>IF(S32=oui,1-S33,1)</f>
         <v>1</v>
       </c>
@@ -2169,7 +2179,7 @@
       <c r="C43" s="50" t="s">
         <v>73</v>
       </c>
-      <c r="D43" s="66">
+      <c r="D43" s="65">
         <f>IF(Elan&lt;=D37,1,IF(Elan&lt;=D38,2,IF(Elan&lt;=D39,3,4)))</f>
         <v>3</v>
       </c>
@@ -2186,14 +2196,14 @@
       <c r="P43" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="Q43" s="64">
+      <c r="Q43" s="63">
         <f>(Nfs*ABS(zANP-tfs/2)+Nfi*ABS(zANP-(Ht-tfi/2))+Nw*hw/2*(pW^2+(1-pW)^2))/1000</f>
         <v>451.07600000000002</v>
       </c>
       <c r="R43" t="s">
         <v>23</v>
       </c>
-      <c r="U43" s="79">
+      <c r="U43" s="78">
         <f>SUM(U39:U42)</f>
         <v>451.07600000000002</v>
       </c>
@@ -2202,6 +2212,16 @@
       <c r="M45" s="56" t="s">
         <v>60</v>
       </c>
+      <c r="P45" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="Q45" s="63">
+        <f>MIN(Nfs,Nfi)*(Ht-(tfs+tfi)/2)/1000</f>
+        <v>372.6</v>
+      </c>
+      <c r="R45" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="46" spans="3:22" x14ac:dyDescent="0.25">
       <c r="M46" s="50" t="s">
@@ -2213,16 +2233,16 @@
       </c>
     </row>
     <row r="48" spans="3:22" x14ac:dyDescent="0.25">
-      <c r="C48" s="68" t="s">
+      <c r="C48" s="67" t="s">
         <v>74</v>
       </c>
-      <c r="D48" s="68"/>
-      <c r="E48" s="68"/>
-      <c r="F48" s="68"/>
-      <c r="G48" s="68"/>
+      <c r="D48" s="67"/>
+      <c r="E48" s="67"/>
+      <c r="F48" s="67"/>
+      <c r="G48" s="67"/>
     </row>
     <row r="50" spans="3:19" x14ac:dyDescent="0.25">
-      <c r="C50" s="67" t="s">
+      <c r="C50" s="66" t="s">
         <v>75</v>
       </c>
       <c r="D50" s="3" t="s">
@@ -2240,6 +2260,9 @@
       <c r="G51" s="4" t="s">
         <v>140</v>
       </c>
+      <c r="I51" s="4" t="s">
+        <v>146</v>
+      </c>
     </row>
     <row r="52" spans="3:19" x14ac:dyDescent="0.25">
       <c r="D52" s="2" t="s">
@@ -2247,14 +2270,18 @@
       </c>
       <c r="E52" s="60">
         <f>ABS(MEd_U1/MRd)</f>
-        <v>0.81057627195071624</v>
+        <v>0.97269152634085954</v>
       </c>
       <c r="F52" s="2" t="s">
         <v>76</v>
       </c>
       <c r="G52" s="60">
         <f>ABS(MEd_U1/MRd)</f>
-        <v>0.81057627195071624</v>
+        <v>0.97269152634085954</v>
+      </c>
+      <c r="I52" s="59">
+        <f>ABS(MEd_U1)/MplRd</f>
+        <v>0.83134549388573098</v>
       </c>
       <c r="M52" s="52" t="s">
         <v>106</v>
@@ -2272,30 +2299,30 @@
       </c>
       <c r="E53" s="60">
         <f>ABS(MEd_U2/MRd)</f>
-        <v>0.56740339036550136</v>
+        <v>0.68088406843860172</v>
       </c>
       <c r="F53" s="2" t="s">
         <v>77</v>
       </c>
       <c r="G53" s="60">
         <f>ABS(MEd_U2/MRd)</f>
-        <v>0.56740339036550136</v>
+        <v>0.68088406843860172</v>
       </c>
     </row>
     <row r="54" spans="3:19" x14ac:dyDescent="0.25">
       <c r="D54" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="E54" s="75">
+      <c r="E54" s="74">
         <f>MAX(E52:E53)</f>
-        <v>0.81057627195071624</v>
+        <v>0.97269152634085954</v>
       </c>
       <c r="F54" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="G54" s="75">
+      <c r="G54" s="74">
         <f>MAX(G52:G53)</f>
-        <v>0.81057627195071624</v>
+        <v>0.97269152634085954</v>
       </c>
       <c r="M54" s="3" t="s">
         <v>107</v>
@@ -2312,7 +2339,7 @@
       <c r="M55" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="N55" s="5">
+      <c r="N55" s="62">
         <f>(bfs^3*tfs+bfi^3*tfi+hw*tw^3)/12/10^4</f>
         <v>1125.2916666666665</v>
       </c>
@@ -2321,10 +2348,10 @@
       </c>
     </row>
     <row r="56" spans="3:19" x14ac:dyDescent="0.25">
-      <c r="C56" s="67" t="s">
+      <c r="C56" s="66" t="s">
         <v>85</v>
       </c>
-      <c r="D56" s="71" t="s">
+      <c r="D56" s="70" t="s">
         <v>86</v>
       </c>
       <c r="E56" s="61">
@@ -2348,13 +2375,13 @@
       </c>
     </row>
     <row r="57" spans="3:19" x14ac:dyDescent="0.25">
-      <c r="E57" s="72" t="s">
+      <c r="E57" s="71" t="s">
         <v>96</v>
       </c>
       <c r="M57" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="N57" s="63">
+      <c r="N57" s="62">
         <f>RhoA*A/(1000)^2</f>
         <v>58.09</v>
       </c>
@@ -2368,12 +2395,12 @@
       </c>
       <c r="E58" s="60">
         <f>VEd_U1/VRd</f>
-        <v>0.56031664323527341</v>
+        <v>0.67237997188232812</v>
       </c>
       <c r="M58" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="N58" s="74">
+      <c r="N58" s="73">
         <f>N57*(LL+La)</f>
         <v>668.03500000000008</v>
       </c>
@@ -2387,7 +2414,7 @@
       </c>
       <c r="E59" s="60">
         <f>VEd_U2/VRd</f>
-        <v>0.39222165026469141</v>
+        <v>0.47066598031762968</v>
       </c>
       <c r="M59" s="3"/>
     </row>
@@ -2395,9 +2422,9 @@
       <c r="D60" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="E60" s="75">
+      <c r="E60" s="74">
         <f>MAX(E58:E59)</f>
-        <v>0.56031664323527341</v>
+        <v>0.67237997188232812</v>
       </c>
       <c r="M60" s="3" t="s">
         <v>115</v>
@@ -2423,7 +2450,7 @@
       </c>
     </row>
     <row r="62" spans="3:19" x14ac:dyDescent="0.25">
-      <c r="C62" s="67" t="s">
+      <c r="C62" s="66" t="s">
         <v>87</v>
       </c>
       <c r="M62" s="3" t="s">
@@ -2481,14 +2508,14 @@
       <c r="N66" s="4"/>
     </row>
     <row r="67" spans="3:18" x14ac:dyDescent="0.25">
-      <c r="M67" s="76" t="s">
+      <c r="M67" s="75" t="s">
         <v>119</v>
       </c>
-      <c r="N67" s="77"/>
-      <c r="O67" s="78"/>
-      <c r="P67" s="78"/>
-      <c r="Q67" s="78"/>
-      <c r="R67" s="78"/>
+      <c r="N67" s="76"/>
+      <c r="O67" s="77"/>
+      <c r="P67" s="77"/>
+      <c r="Q67" s="77"/>
+      <c r="R67" s="77"/>
     </row>
     <row r="68" spans="3:18" x14ac:dyDescent="0.25">
       <c r="D68" s="50" t="s">
@@ -2505,16 +2532,16 @@
       <c r="D69" s="50" t="s">
         <v>93</v>
       </c>
-      <c r="E69" s="73">
+      <c r="E69" s="72">
         <f>ElancementW/(37.4*EpsilonW*SQRT(kTau))</f>
         <v>0.90654795175087832</v>
       </c>
       <c r="M69" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="N69" s="61">
+      <c r="N69" s="62">
         <f>-qQ_1*La^2*LL^2/18/SQRT(3)/(E*InertieCM4/100)*1000^2</f>
-        <v>-53.961851440791989</v>
+        <v>-64.754221728950398</v>
       </c>
       <c r="O69" t="s">
         <v>7</v>
@@ -2531,9 +2558,9 @@
       <c r="M70" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="N70" s="61">
+      <c r="N70" s="62">
         <f>qQ_1*La^3/24/(E*InertieCM4/100)*1000^2*(4*LL+3*La)</f>
-        <v>94.113728562921224</v>
+        <v>112.93647427550546</v>
       </c>
       <c r="O70" t="s">
         <v>7</v>
@@ -2552,8 +2579,11 @@
       </c>
     </row>
     <row r="73" spans="3:18" x14ac:dyDescent="0.25">
-      <c r="E73" s="72" t="s">
+      <c r="E73" s="71" t="s">
         <v>96</v>
+      </c>
+      <c r="G73" s="4" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="74" spans="3:18" x14ac:dyDescent="0.25">
@@ -2562,7 +2592,11 @@
       </c>
       <c r="E74" s="60">
         <f>VEd_U1/VbRd</f>
-        <v>0.73439118832317785</v>
+        <v>0.88126942598781344</v>
+      </c>
+      <c r="G74" s="59">
+        <f>IF(ABS(MEd_Q1)&gt;MfRd,ABS(MEd_U1)/MplRd+(1-MfRd/MplRd)*(2*E74-1)^2,0)</f>
+        <v>0.93250602257403981</v>
       </c>
     </row>
     <row r="75" spans="3:18" x14ac:dyDescent="0.25">
@@ -2571,25 +2605,30 @@
       </c>
       <c r="E75" s="60">
         <f>VEd_U2/VbRd</f>
-        <v>0.51407383182622446</v>
-      </c>
+        <v>0.61688859819146946</v>
+      </c>
+      <c r="G75" s="4"/>
     </row>
     <row r="76" spans="3:18" x14ac:dyDescent="0.25">
       <c r="D76" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="E76" s="75">
+      <c r="E76" s="74">
         <f>MAX(E74:E75)</f>
-        <v>0.73439118832317785</v>
+        <v>0.88126942598781344</v>
+      </c>
+      <c r="G76" s="79">
+        <f>G74</f>
+        <v>0.93250602257403981</v>
       </c>
     </row>
     <row r="78" spans="3:18" x14ac:dyDescent="0.25">
-      <c r="C78" s="67" t="s">
+      <c r="C78" s="66" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="79" spans="3:18" x14ac:dyDescent="0.25">
-      <c r="D79" s="71" t="s">
+      <c r="D79" s="70" t="s">
         <v>98</v>
       </c>
       <c r="E79" s="61">
@@ -2611,7 +2650,7 @@
       </c>
       <c r="E81" s="62">
         <f>VEd_U1*(MStatS/InertieCM4)*100</f>
-        <v>762.99301023944349</v>
+        <v>915.59161228733217</v>
       </c>
       <c r="F81" t="s">
         <v>12</v>
@@ -2623,7 +2662,7 @@
       </c>
       <c r="E82" s="62">
         <f>VEd_U2*(MStatS/InertieCM4)*100</f>
-        <v>534.09510716761042</v>
+        <v>640.91412860113257</v>
       </c>
       <c r="F82" t="s">
         <v>12</v>
@@ -2643,7 +2682,7 @@
       </c>
       <c r="E85" s="60">
         <f>E81/Fu*GammaM2*SQRT(3)/2*BetaW</f>
-        <v>1.58163350212656</v>
+        <v>1.897960202551872</v>
       </c>
       <c r="F85" t="s">
         <v>7</v>
@@ -2655,14 +2694,14 @@
       </c>
       <c r="E86" s="60">
         <f>E82/Fu*GammaM2*SQRT(3)/2*BetaW</f>
-        <v>1.1071434514885918</v>
+        <v>1.3285721417863103</v>
       </c>
       <c r="F86" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="89" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C89" s="67" t="s">
+      <c r="C89" s="66" t="s">
         <v>123</v>
       </c>
     </row>
@@ -2671,7 +2710,7 @@
         <v>124</v>
       </c>
       <c r="E90" s="5">
-        <v>4189</v>
+        <v>277.3</v>
       </c>
       <c r="F90" t="s">
         <v>23</v>
@@ -2683,7 +2722,7 @@
       </c>
       <c r="E91" s="59">
         <f>SQRT(MRd*GammaM0/Mcr)</f>
-        <v>0.30337017873021627</v>
+        <v>1.1791067696894353</v>
       </c>
     </row>
     <row r="92" spans="3:6" x14ac:dyDescent="0.25">
@@ -2700,16 +2739,16 @@
       </c>
       <c r="E93" s="60">
         <f>0.5*(1+AlphaLT*(LambdaLT-0.2)+LambdaLT^2)</f>
-        <v>0.58529740058888391</v>
+        <v>1.5672069596457128</v>
       </c>
     </row>
     <row r="94" spans="3:6" x14ac:dyDescent="0.25">
       <c r="D94" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="E94" s="69">
+      <c r="E94" s="68">
         <f>1/(PhiLT+SQRT(PhiLT^2-LambdaLT^2))</f>
-        <v>0.92094880177136085</v>
+        <v>0.38467388519331625</v>
       </c>
     </row>
     <row r="95" spans="3:6" x14ac:dyDescent="0.25">
@@ -2718,7 +2757,7 @@
       </c>
       <c r="E95" s="62">
         <f>KhiLT*MRd*GammaM0/GammaM1</f>
-        <v>355.05172124141393</v>
+        <v>148.30262528363306</v>
       </c>
       <c r="F95" t="s">
         <v>23</v>
@@ -2732,9 +2771,9 @@
       <c r="D97" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="E97" s="75">
+      <c r="E97" s="74">
         <f>MEd_U1/E95</f>
-        <v>-0.88015345738182948</v>
+        <v>-2.5286133625942337</v>
       </c>
     </row>
     <row r="98" spans="4:5" x14ac:dyDescent="0.25">

</xml_diff>